<commit_message>
Update preliminary submission pack: revised tech report exports, offline verification, and code package.
Sync review fixes into the report Markdown/DOCX/PDF pipeline, refresh designated-set offline materials, and repack the XH-202610 source bundle for GitHub backup.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
@@ -215,7 +215,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>11</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3619500"/>
@@ -240,7 +240,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>31</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3629025"/>
@@ -265,7 +265,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>51</row>
+      <row>54</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="4819650"/>
@@ -290,7 +290,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>71</row>
+      <row>74</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6096000" cy="3629025"/>
@@ -613,7 +613,7 @@
     <col width="23.2" customWidth="1" min="5" max="5"/>
     <col width="35.2" customWidth="1" min="6" max="6"/>
     <col width="21.4" customWidth="1" min="7" max="7"/>
-    <col width="28.4" customWidth="1" min="8" max="8"/>
+    <col width="35.2" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -699,7 +699,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>原始/nested_N0_metrics.json</t>
+          <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>测试集 S07/S08 共 120 trial、无标签：盲测预测见 原始/submission_QuadFold59.csv；未使用测试标签调参，故准/召/特以 train 嵌套主读为准。</t>
+          <t>测试集 S07/S08 共 120 trial、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准/召/特以 train 嵌套主读为准。</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始/nested_N0_metrics.json 与 原始/oof_N0/。</t>
+          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="67.80000000000004" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="70.60000000000002" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -1663,7 +1663,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始/官方数据说明.md。</t>
+          <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始验证数据/官方数据说明.md。</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
     <col width="39.40000000000001" customWidth="1" min="3" max="3"/>
-    <col width="35.3" customWidth="1" min="4" max="4"/>
+    <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>原始/nested_N0_metrics.json</t>
+          <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
@@ -1742,16 +1742,16 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>盲测交卷预测 CSV（120 行）</t>
+          <t>盲测交卷预测 CSV（官方模板已填 label）</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>原始/submission_QuadFold59.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
+          <t>原始验证数据/sample_submission.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
           <t>D3</t>
@@ -1759,12 +1759,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>官方提交模板（行序对照）</t>
+          <t>同内容内部备份（模型名归档）</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>原始/sample_submission.csv</t>
+          <t>原始验证数据/submission_QuadFold59.csv</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>原始/oof_N0/oof_N0_*.npy</t>
+          <t>原始验证数据/oof_N0/oof_N0_*.npy</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>原始/官方数据说明.md</t>
+          <t>原始验证数据/官方数据说明.md</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>原始/数据说明_使用对照.md</t>
+          <t>原始验证数据/数据说明_使用对照.md</t>
         </is>
       </c>
     </row>
@@ -1832,11 +1832,11 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>截图/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="38" customHeight="1">
+          <t>验证过程截图/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
       <c r="B12" s="6" t="inlineStr">
         <is>
           <t>D8</t>
@@ -1875,13 +1875,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F10"/>
+  <dimension ref="A2:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="43.1" customWidth="1" min="2" max="2"/>
-    <col width="30.49999999999999" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1925,12 +1925,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>指定集目录与 PKL 结构核验</t>
+          <t>指定集官方数据核验：目录树、PKL 结构（data 64×22500、ch_names、srate=250）、train 900 / test 120 计数（终端回放）</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>截图/S01_指定集目录与pkl结构.png</t>
+          <t>验证过程截图/S01_数据集结构与加载核验.png</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1947,12 +1947,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>嵌套 N0 主读 Acc/召/特/F1 汇总</t>
+          <t>嵌套 N0 主读回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>截图/S02_嵌套N0指标汇总.png</t>
+          <t>验证过程截图/S02_嵌套N0指标汇总.png</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>交卷 CSV 前 30 行与标签分布</t>
+          <t>盲测交卷 CSV 再生成与比对：predict_submission.py 现场重生成，与交稿 CSV 逐行 diff（终端回放）</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>截图/S03_交卷CSV前30行.png</t>
+          <t>验证过程截图/S03_交卷CSV再生成与比对.png</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1991,12 +1991,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>核心指标填写说明（准/召/特/延迟）</t>
+          <t>指定集指标独立复算：从 OOF npy 重算 Acc/召/特/F1/CM/六折，逐项对照登记 JSON（终端回放）</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>截图/S04_Excel总表指定集行说明.png</t>
+          <t>验证过程截图/S04_独立复算.png</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -2005,11 +2005,77 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>下列嵌入图便于审阅；原图亦在交稿/验证过程截图/。</t>
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>交卷 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>验证过程截图/S05_交卷CSV完整性校验.png</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>S06</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Excel 核心指标与登记 JSON 一致性：程序化读取 00 表单元格对照（终端回放）</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>验证过程截图/S06_Excel与JSON一致性.png</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>交稿包文件 MD5 指纹与运行环境（python/numpy 版本、时间戳；终端回放）</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>验证过程截图/S07_文件指纹与环境.png</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>下列嵌入图便于审阅；原图亦在交稿包 验证过程截图/ 目录。</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2158,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>submission_QuadFold59.csv（120 行，label∈{0,1,2}）</t>
+          <t>sample_submission.csv（官方模板已填 label∈{0,1,2}，120 行）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync preliminary materials and report assets with latest offline pack and figures.
Include revised tech report drafts/figures, offline verification pack updates, code package refresh, and Leave-Next tooling; keep submission numbers unchanged.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22320" windowHeight="11480" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_核心指标" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_数据核对" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,41 +26,197 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="26">
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <color rgb="001B2A4A"/>
+      <charset val="134"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <color rgb="008C8A84"/>
+      <charset val="134"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Noto Sans SC"/>
+      <charset val="134"/>
+      <color rgb="FF37352F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Noto Sans SC"/>
+      <charset val="134"/>
+      <color rgb="FF8C8A84"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <color rgb="00FFFFFF"/>
+      <charset val="134"/>
+      <color rgb="FF1B2A4A"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
-      <color rgb="0037352F"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
-      <color rgb="001B2A4A"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
       <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill/>
     </fill>
@@ -70,21 +225,210 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B2A4A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7F7F5"/>
+        <fgColor rgb="FF1B2A4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -93,49 +437,358 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="00E9E9E8"/>
+        <color rgb="FFE9E9E8"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -218,7 +871,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="3619500"/>
+    <ext cx="8572500" cy="3190875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -240,10 +893,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>34</row>
+      <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="3629025"/>
+    <ext cx="8572500" cy="4219575"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -265,10 +918,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>54</row>
+      <row>58</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="4819650"/>
+    <ext cx="8572500" cy="2333625"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -290,10 +943,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>74</row>
+      <row>73</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6096000" cy="3629025"/>
+    <ext cx="8572500" cy="2943225"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -301,6 +954,81 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>91</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="1885950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>103</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="2009775"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>116</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="3476625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -593,7 +1321,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -603,8 +1330,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
@@ -625,223 +1352,223 @@
       </c>
     </row>
     <row r="3" ht="8" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>本报告仅报告主办方指定标准脑电数据集（Challenge MI / S01–S08）上的算法性能；不含自采数据与其他公开库读数。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>指标（官方要求）</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>模型</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>评测协议</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>评测方案</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>样本规模</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>证据文件</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>分类准确率</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="14" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>三分类试次级 Acc；类均衡下与 macro 召回同值</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>LOSO6 · leave-fold 嵌套 Val（主读）</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>900 trial（S01–S06）</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折（LOSO6）· 嵌套验证集（主要结果）</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>900 试次（S01–S06）</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>召回率（macro）</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>三类召回率算术平均</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>每类 300 trial</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>每类 300 试次</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>特异性（macro）</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="14" t="n">
         <v>0.7556</v>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>三类特异性算术平均</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>运算延迟（单 trial 前向）</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>运算延迟（单试次前向）</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>RTX 5070；3 s / 750 点窗；四成员融合链路单窗增量</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>QuadFold-59（同构推理）</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>离线批推理计时</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>单窗</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>sheet 03</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>判定延迟（协议上界）</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>判定延迟（实验范式时序上界）</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>指定集 1 trial = 1 窗（750 点）；无滑窗 hop；+前向 1.11 ms</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>指定集 1 试次 = 1 窗（750 点）；无滑窗步长；+前向 1.11 ms</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>官方 trial 切分</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>单 trial</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>官方试次切分</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>单试次</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>sheet 03 · 官方数据说明</t>
         </is>
@@ -849,23 +1576,23 @@
     </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>附报（不作主读）：折内 Val Acc=0.558±0.069（融合参数本折拟合，乐观偏置约 +4.7 pp）。</t>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>附报（不作主要结果）：折内验证准确率 0.5580 ± 0.0690（融合参数在本折内拟合，存在约 4.7 个百分点的乐观偏置）。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>测试集 S07/S08 共 120 trial、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准/召/特以 train 嵌套主读为准。</t>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>测试集 S07/S08 共 120 试次、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准确率/召回率/特异性以训练集嵌套验证的主要结果为准。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>交卷模型：QuadFold-59 = 59 EEG 通道、从零训练的四成员温度校准集成（内部代号 S0 / E1f-A59）。</t>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>提交模型：QuadFold-59 = 59 通道脑电、从零训练的四成员温度校准集成。</t>
         </is>
       </c>
     </row>
@@ -883,17 +1610,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="3" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -906,39 +1628,39 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>支持数</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>召回率</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>特异性</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>精确率</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>左手运动想象 / Left(0)</t>
         </is>
@@ -946,43 +1668,43 @@
       <c r="C5" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.3267</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="14" t="n">
         <v>0.85</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="14" t="n">
         <v>0.5213</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="14" t="n">
         <v>0.4016</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>右手运动想象 / Right(1)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.6233</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.7117</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="15" t="n">
         <v>0.5194</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="15" t="n">
         <v>0.5667</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>静息态（空闲） / Rest(2)</t>
         </is>
@@ -990,69 +1712,69 @@
       <c r="C7" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.5833</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="14" t="n">
         <v>0.705</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="14" t="n">
         <v>0.4972</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="14" t="n">
         <v>0.5368000000000001</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>macro / 总体</t>
         </is>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.7556</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="15" t="n">
         <v>0.5125999999999999</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="15" t="n">
         <v>0.5017</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>混淆矩阵（行=真实，列=预测；类序 左 / 右 / 静息）</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>预测·左手</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>预测·右手</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>预测·静息</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>真实·左手</t>
         </is>
@@ -1068,23 +1790,23 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>真实·右手</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="7" t="n">
         <v>46</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="7" t="n">
         <v>67</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>真实·静息</t>
         </is>
@@ -1101,9 +1823,9 @@
     </row>
     <row r="15" ht="22" customHeight="1"/>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>来源：嵌套验证折外预测（OOF）概率逐试次取最大类别；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
         </is>
       </c>
     </row>
@@ -1122,17 +1844,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="29.09999999999999" customWidth="1" min="6" max="6"/>
+    <col width="29.1" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="10" t="n"/>
+    </row>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1142,37 +1865,37 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="38" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>折</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>保留被试（Val）</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Val 试次数</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>嵌套 Acc</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
@@ -1180,41 +1903,41 @@
       <c r="D5" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="14" t="n">
         <v>0.4267</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="15" t="n">
         <v>0.62</v>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
@@ -1222,41 +1945,41 @@
       <c r="D7" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="14" t="n">
         <v>0.5467</v>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>S04</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="15" t="n">
         <v>0.4867</v>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
@@ -1264,43 +1987,43 @@
       <c r="D9" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="14" t="n">
         <v>0.4867</v>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="7" t="n">
         <v>150</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="15" t="n">
         <v>0.5</v>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折 OOF 上拟合</t>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>S01–S06</t>
         </is>
@@ -1308,12 +2031,12 @@
       <c r="D11" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>0.5111 ± 0.0657</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>主报表 mean±std（ddof=1）</t>
         </is>
@@ -1321,9 +2044,9 @@
     </row>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>划分：每折 Train=750 trial / Val=150 trial；禁止随机 Val；Test=S07–S08 不参与调参。</t>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>划分：每折训练集 750 试次 / 验证集 150 试次；禁止随机验证集；测试集 S07–S08 不参与调参。</t>
         </is>
       </c>
     </row>
@@ -1341,131 +2064,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="25.7" customWidth="1" min="3" max="3"/>
-    <col width="45.40000000000001" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="45.4" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>指定集协议下的运算延迟与判定延迟</t>
+          <t>指定集实验范式下的运算延迟与判定延迟</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>单 trial / 单窗前向（四成员融合）</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>单试次 / 单窗前向（四成员融合）</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>RTX 5070；输入 (1,1,59,750) 同构链路实测口径</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>已实测</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>采样与窗长</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>250 Hz · 750 点 = 3.00 s</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>与官方《数据说明》一致；1 trial = 1 窗</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>协议冻结</t>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>与官方《数据说明》一致；1 试次 = 1 窗</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>官方冻结</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>判定延迟（指定集离线）</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>3.00 s + 1.11 ms</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>积累满 3 s trial 后给出类别；无 100 ms 滑窗 hop</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>协议上界</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>积累满 3 s 试次后给出类别；无 100 ms 滑窗步长</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>范式上界</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>在线系统对照（非本表主读）</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>在线系统对照（非本表主要结果）</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>判定约 3.5 s</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>仅说明同栈在线节拍；本 Excel 主读为指定集离线</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>仅说明同栈在线节拍；本 Excel 主要结果为指定集离线口径</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>附注</t>
         </is>
@@ -1473,9 +2195,9 @@
     </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>官方核心量化指标中的「运算延迟」取单 trial 前向 1.11 ms；「判定延迟」取协议窗长 3.00 s。</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>官方核心量化指标中的「运算延迟」取单试次前向 1.11 ms；「判定延迟」取实验范式窗长 3.00 s。</t>
         </is>
       </c>
     </row>
@@ -1493,17 +2215,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="72" customWidth="1" min="2" max="2"/>
-    <col width="70.60000000000002" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="70.59999999999999" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1516,144 +2234,144 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>数据集名称</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>主办方指定标准脑电数据集（Challenge MI）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>数据路径</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>DATA/挑战杯运动想象赛题数据文件/</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>3 s EEG trial → 三类：0 左手(201) / 1 右手(202) / 2 静息(204)</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>每试次 3 s 脑电 → 三类：0 左手(201) / 1 右手(202) / 2 静息(204)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>训练集</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>S01–S06 × 各 5 block × 30 trial = 900 trial（三类各 300）</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>S01–S06 × 各 5 数据块 × 30 试次 = 900 试次（三类各 300）</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>测试集</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>S07–S08 × 各 2 block × 30 trial = 120 trial（无 trigger / 无标签）</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>S07–S08 × 各 2 数据块 × 30 试次 = 120 试次（无 trigger / 无标签）</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>采样率 / 窗</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>250 Hz；每 trial 750 点；起点 0,750,…,21750</t>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>250 Hz；每试次 750 点；起点 0,750,…,21750</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>通道</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>64 信号中取 59 EEG（丢弃 ECG, HEOR, HEOL, VEOU, VEOL）；训练测试通道序一致</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>64 信号通道中取 59 个脑电通道（丢弃 ECG、HEOR、HEOL、VEOU、VEOL）；训练与测试通道顺序一致</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>预处理硬约束</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>先按 trial 切分，再滤波/标准化；可学习统计量仅用该折 Train 拟合</t>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>先按试次切分，再滤波/标准化；可学习统计量仅用该折训练集拟合</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>划分与主读</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>LOSO6；主读=leave-fold 嵌套 Val Acc/召/特；折内仅附报</t>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>划分与主要结果</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折（LOSO6）；主要结果 = 逐折嵌套验证集 Acc/召/特；折内读数仅附报</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>交卷模型</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>QuadFold-59（59ch 从零四成员集成）；盲测 CSV 对齐 sample_submission.csv</t>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>提交模型</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>QuadFold-59（59 通道从零训练四成员集成）；盲测 CSV 与官方模板 sample_submission.csv 逐行对齐</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>未使用</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>未使用测试集标签调参；本报告不含自采数据指标</t>
         </is>
@@ -1661,7 +2379,7 @@
     </row>
     <row r="16" ht="22" customHeight="1"/>
     <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始验证数据/官方数据说明.md。</t>
         </is>
@@ -1681,12 +2399,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="39.40000000000001" customWidth="1" min="3" max="3"/>
+    <col width="39.4" customWidth="1" min="3" max="3"/>
     <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1701,153 +2419,153 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>相对路径</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>嵌套主读指标 JSON（Acc/召/特/F1/CM/六折）</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>嵌套主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>嵌套主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>盲测交卷预测 CSV（官方模板已填 label）</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>盲测提交预测 CSV（官方模板已填 label）</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>原始验证数据/sample_submission.csv</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>同内容内部备份（模型名归档）</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/submission_QuadFold59.csv</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>嵌套 OOF 概率 / 标签 / 被试</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>原始验证数据/oof_N0/oof_N0_*.npy</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>官方《数据说明》副本</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>原始验证数据/官方数据说明.md</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>本队使用对照摘录</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>原始验证数据/数据说明_使用对照.md</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>验证过程截图 S01–S04</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>验证过程截图/</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>交稿包（邮件附件）</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>交稿/ 或 交稿_离线验证_XH-202610.zip</t>
         </is>
@@ -1855,7 +2573,7 @@
     </row>
     <row r="13" ht="22" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>复算嵌套指标：对 oof_N0_prob.npy 做 argmax，与 oof_N0_y.npy 对照即可复现 sheet 00/01/02。</t>
         </is>
@@ -1875,15 +2593,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="2" max="3"/>
     <col width="38.2" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="5" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1896,186 +2612,192 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>文件</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>指定集官方数据核验：目录树、PKL 结构（data 64×22500、ch_names、srate=250）、train 900 / test 120 计数（终端回放）</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>验证过程截图/S01_数据集结构与加载核验.png</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>嵌套 N0 主读回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>嵌套验证主结果回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>验证过程截图/S02_嵌套N0指标汇总.png</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>盲测交卷 CSV 再生成与比对：predict_submission.py 现场重生成，与交稿 CSV 逐行 diff（终端回放）</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>验证过程截图/S03_交卷CSV再生成与比对.png</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>盲测提交 CSV 再生成与比对：predict_submission.py 现场重生成，与提交 CSV 逐行比对（终端回放）</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>验证过程截图/S03_提交CSV再生成与比对.png</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>S04</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>指定集指标独立复算：从 OOF npy 重算 Acc/召/特/F1/CM/六折，逐项对照登记 JSON（终端回放）</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>验证过程截图/S04_独立复算.png</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>交卷 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>验证过程截图/S05_交卷CSV完整性校验.png</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>提交 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>验证过程截图/S05_提交CSV完整性校验.png</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Excel 核心指标与登记 JSON 一致性：程序化读取 00 表单元格对照（终端回放）</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>验证过程截图/S06_Excel与JSON一致性.png</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>交稿包文件 MD5 指纹与运行环境（python/numpy 版本、时间戳；终端回放）</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>验证过程截图/S07_文件指纹与环境.png</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="B13" s="2" t="inlineStr">
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>下列嵌入图便于审阅；原图亦在交稿包 验证过程截图/ 目录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>注：S07 中 xlsx 自身 MD5 为嵌入本截图前一版的指纹（自引用无法自洽）；交稿包核验以 S07 其余 13 项文件指纹为准。</t>
         </is>
       </c>
     </row>
@@ -2094,95 +2816,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="15.6" customWidth="1" min="2" max="2"/>
-    <col width="63.60000000000002" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="63.6" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>交卷决策与评测纪律（指定集）</t>
+          <t>提交决策与评测纪律（指定集）</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>项</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>交卷模型</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>QuadFold-59（嵌套主读 0.511±0.066）</t>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>提交模型</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>QuadFold-59（嵌套主要结果 0.5111 ± 0.0657）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>主读尺子</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>LOSO6 leave-fold 嵌套；禁止用折内 0.558 作对外主读</t>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>主要结果口径</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折嵌套；折内 0.5580 仅内部参考，不作为对外报告结果</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>盲测文件</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>sample_submission.csv（官方模板已填 label∈{0,1,2}，120 行）</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>风险否决（归档）</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>备选 8ch 微调栈嵌套 0.540：test 预测 Rest≈51% 落在 Val 支撑外，不交</t>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>备选 8 通道微调方案嵌套 0.540：测试集预测静息类占比约 51%，超出验证集支撑范围，不提交</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>纪律</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>超参与融合权仅在 Val/嵌套折外选定；测试标签未用于调参</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>超参数与融合权重仅在验证集/嵌套折外选定；测试集标签未用于调参</t>
         </is>
       </c>
     </row>
@@ -2200,15 +2920,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="B2:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="3" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -2221,145 +2938,145 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>核对项</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>期望</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>表内</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>准确率</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="14" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>召回率 macro</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>特异性 macro</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="14" t="n">
         <v>0.7556</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.7556</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>运算延迟</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>判定延迟（指定集）</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>OOF 试次数</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="7" t="n">
         <v>900</v>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>盲测 CSV 行数</t>
         </is>
@@ -2370,29 +3087,29 @@
       <c r="D11" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>本报告是否含自采指标</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>

<commit_message>
Sync contest materials and tighten GitHub ignore for large media.
Exclude videos, archives, DATA caches, and the submission bundle so pushes stay within GitHub size limits while keeping source and report assets.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
+++ b/资料/初赛材料/02_离线验证/交稿/离线性能验证报告_XH-202610.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22320" windowHeight="11480" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_核心指标" sheetId="1" state="visible" r:id="rId1"/>
@@ -13,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_数据集使用说明" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_原始数据索引" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_验证过程截图" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_交卷与评测纪律" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_提交决策与评测纪律" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_数据核对" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,197 +27,41 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="6">
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <charset val="134"/>
-      <color rgb="FF1B2A4A"/>
+      <color rgb="001B2A4A"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <charset val="134"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="008C8A84"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Noto Sans SC"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <charset val="134"/>
-      <color rgb="FF37352F"/>
+      <color rgb="0037352F"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Noto Sans SC"/>
-      <charset val="134"/>
-      <color rgb="FF8C8A84"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Noto Sans SC"/>
-      <charset val="134"/>
-      <color rgb="FF1B2A4A"/>
+      <color rgb="001B2A4A"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -225,210 +70,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1B2A4A"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="001B2A4A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF7F7F5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="00F7F7F5"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -437,358 +93,49 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="thin">
-        <color rgb="FFE9E9E8"/>
+        <color rgb="00E9E9E8"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -871,7 +218,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="3190875"/>
+    <ext cx="6096000" cy="2266950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -893,10 +240,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>33</row>
+      <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="4219575"/>
+    <ext cx="6096000" cy="3000375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -918,10 +265,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>58</row>
+      <row>50</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="2333625"/>
+    <ext cx="6096000" cy="1657350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -943,10 +290,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>73</row>
+      <row>68</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="2943225"/>
+    <ext cx="6096000" cy="2085975"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -968,10 +315,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>91</row>
+      <row>86</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="1885950"/>
+    <ext cx="6096000" cy="1333500"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -993,10 +340,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>103</row>
+      <row>104</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="2009775"/>
+    <ext cx="6096000" cy="1428750"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -1018,10 +365,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>116</row>
+      <row>122</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8572500" cy="3476625"/>
+    <ext cx="6096000" cy="2466975"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -1321,6 +668,7 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1330,16 +678,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="23.2" customWidth="1" min="5" max="5"/>
-    <col width="35.2" customWidth="1" min="6" max="6"/>
-    <col width="21.4" customWidth="1" min="7" max="7"/>
+    <col width="37.2" customWidth="1" min="6" max="6"/>
+    <col width="19.8" customWidth="1" min="7" max="7"/>
     <col width="35.2" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1352,223 +700,223 @@
       </c>
     </row>
     <row r="3" ht="8" customHeight="1">
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>本报告仅报告主办方指定标准脑电数据集（Challenge MI / S01–S08）上的算法性能；不含自采数据与其他公开库读数。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>指标（官方要求）</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>模型</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>评测方案</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>评测协议</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>样本规模</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>证据文件</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>分类准确率</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="5" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>三分类试次级 Acc；类均衡下与 macro 召回同值</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>留一被试交叉验证 6 折（LOSO6）· 嵌套验证集（主要结果）</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折（LOSO6）；主要结果</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>900 试次（S01–S06）</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>召回率（macro）</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="7" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>三类召回率算术平均</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>每类 300 试次</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>特异性（macro）</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="5" t="n">
         <v>0.7556</v>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>三类特异性算术平均</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>同上</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>运算延迟（单试次前向）</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>运算延迟（单 trial 前向）</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>RTX 5070；3 s / 750 点窗；四成员融合链路单窗增量</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>QuadFold-59（同构推理）</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>离线批推理计时</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>单窗</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>sheet 03</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>判定延迟（实验范式时序上界）</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>判定延迟（协议上界）</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>指定集 1 试次 = 1 窗（750 点）；无滑窗步长；+前向 1.11 ms</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>指定集 1 trial = 1 窗（750 点）；无滑窗 hop；+前向 1.11 ms</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>QuadFold-59</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>官方试次切分</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>单试次</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>官方 trial 切分</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>单 trial</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>sheet 03 · 官方数据说明</t>
         </is>
@@ -1576,23 +924,23 @@
     </row>
     <row r="11" ht="22" customHeight="1"/>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>附报（不作主要结果）：折内验证准确率 0.5580 ± 0.0690（融合参数在本折内拟合，存在约 4.7 个百分点的乐观偏置）。</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>附报（不作主要结果）：折内验证准确率 0.5580 ± 0.0690（融合参数在本折拟合，乐观偏置约 +4.7 个百分点）。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>测试集 S07/S08 共 120 试次、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准确率/召回率/特异性以训练集嵌套验证的主要结果为准。</t>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>测试集 S07/S08 共 120 试次、无标签：盲测预测已写入官方模板 原始验证数据/sample_submission.csv；未使用测试标签调参，故准/召/特以训练集留一被试主要结果为准。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>提交模型：QuadFold-59 = 59 通道脑电、从零训练的四成员温度校准集成。</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>提交模型：QuadFold-59 = 59 EEG 通道、从零训练的四成员温度校准集成。</t>
         </is>
       </c>
     </row>
@@ -1610,12 +958,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="8"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1628,39 +981,39 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>类别</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>支持数</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>召回率</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>特异性</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>精确率</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>F1</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>左手运动想象 / Left(0)</t>
         </is>
@@ -1668,43 +1021,43 @@
       <c r="C5" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.3267</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.5213</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="5" t="n">
         <v>0.4016</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>右手运动想象 / Right(1)</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.6233</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.7117</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="7" t="n">
         <v>0.5194</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="7" t="n">
         <v>0.5667</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>静息态（空闲） / Rest(2)</t>
         </is>
@@ -1712,69 +1065,69 @@
       <c r="C7" s="8" t="n">
         <v>300</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="5" t="n">
         <v>0.5833</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="5" t="n">
         <v>0.705</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.4972</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="5" t="n">
         <v>0.5368000000000001</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>macro / 总体</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="9" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="7" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="7" t="n">
         <v>0.7556</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="7" t="n">
         <v>0.5125999999999999</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="7" t="n">
         <v>0.5017</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>混淆矩阵（行=真实，列=预测；类序 左 / 右 / 静息）</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="2" t="inlineStr"/>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>预测·左手</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>预测·右手</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>预测·静息</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>真实·左手</t>
         </is>
@@ -1790,23 +1143,23 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>真实·右手</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="9" t="n">
         <v>46</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="9" t="n">
         <v>187</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="9" t="n">
         <v>67</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>真实·静息</t>
         </is>
@@ -1823,9 +1176,9 @@
     </row>
     <row r="15" ht="22" customHeight="1"/>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>来源：嵌套验证折外预测（OOF）概率逐试次取最大类别；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>来源：Exp37 nested-S0（N0）OOF 概率 argmax；文件 原始验证数据/nested_N0_metrics.json 与 原始验证数据/oof_N0/。</t>
         </is>
       </c>
     </row>
@@ -1844,18 +1197,17 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="29.1" customWidth="1" min="6" max="6"/>
+    <col width="29.09999999999999" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="10" t="n"/>
-    </row>
+    <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1865,37 +1217,37 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="38" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>折</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>保留被试（Val）</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Val 试次数</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>嵌套 Acc</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
@@ -1903,41 +1255,41 @@
       <c r="D5" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="5" t="n">
         <v>0.4267</v>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折 OOF 上拟合</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="7" t="n">
         <v>0.62</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折 OOF 上拟合</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
@@ -1945,41 +1297,41 @@
       <c r="D7" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="5" t="n">
         <v>0.5467</v>
       </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折 OOF 上拟合</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>S04</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="7" t="n">
         <v>0.4867</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折 OOF 上拟合</t>
         </is>
       </c>
     </row>
     <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
@@ -1987,43 +1339,43 @@
       <c r="D9" s="8" t="n">
         <v>150</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="5" t="n">
         <v>0.4867</v>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折 OOF 上拟合</t>
         </is>
       </c>
     </row>
     <row r="10" ht="38" customHeight="1">
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>融合参数仅在其余五折的折外预测（OOF）上拟合</t>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>融合参数仅在其余五折 OOF 上拟合</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>S01–S06</t>
         </is>
@@ -2031,12 +1383,12 @@
       <c r="D11" s="8" t="n">
         <v>900</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>0.5111 ± 0.0657</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>主报表 mean±std（ddof=1）</t>
         </is>
@@ -2044,9 +1396,9 @@
     </row>
     <row r="12" ht="22" customHeight="1"/>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>划分：每折训练集 750 试次 / 验证集 150 试次；禁止随机验证集；测试集 S07–S08 不参与调参。</t>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>划分：每折 Train=750 trial / Val=150 trial；禁止随机 Val；Test=S07–S08 不参与调参。</t>
         </is>
       </c>
     </row>
@@ -2064,130 +1416,131 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="25.7" customWidth="1" min="3" max="3"/>
-    <col width="45.4" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="6"/>
+    <col width="45.40000000000001" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>指定集实验范式下的运算延迟与判定延迟</t>
+          <t>指定集协议下的运算延迟与判定延迟</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>数值</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>单试次 / 单窗前向（四成员融合）</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>单 trial / 单窗前向（四成员融合）</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>RTX 5070；输入 (1,1,59,750) 同构链路实测口径</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>已实测</t>
         </is>
       </c>
     </row>
     <row r="6" ht="38" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>采样与窗长</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>250 Hz · 750 点 = 3.00 s</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>与官方《数据说明》一致；1 试次 = 1 窗</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>官方冻结</t>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>与官方《数据说明》一致；1 trial = 1 窗</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>协议冻结</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>判定延迟（指定集离线）</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>3.00 s + 1.11 ms</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>积累满 3 s 试次后给出类别；无 100 ms 滑窗步长</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>范式上界</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>积累满 3 s trial 后给出类别；无 100 ms 滑窗 hop</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>协议上界</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>在线系统对照（非本表主要结果）</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>在线系统对照（非本表主读）</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>判定约 3.5 s</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>仅说明同栈在线节拍；本 Excel 主要结果为指定集离线口径</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>仅说明同栈在线节拍；本 Excel 主读为指定集离线</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>附注</t>
         </is>
@@ -2195,9 +1548,9 @@
     </row>
     <row r="9" ht="22" customHeight="1"/>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>官方核心量化指标中的「运算延迟」取单试次前向 1.11 ms；「判定延迟」取实验范式窗长 3.00 s。</t>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>官方核心量化指标中的「运算延迟」取单 trial 前向 1.11 ms；「判定延迟」取协议窗长 3.00 s。</t>
         </is>
       </c>
     </row>
@@ -2215,173 +1568,189 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="72" customWidth="1" min="2" max="2"/>
-    <col width="70.59999999999999" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="8"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>数据集使用说明（仅主办方指定标准数据集）</t>
+          <t>数据集使用说明（仅主办方指定标准数据集 · Excel 正文）</t>
         </is>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>数据集名称</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>主办方指定标准脑电数据集（Challenge MI）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>数据路径</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>DATA/挑战杯运动想象赛题数据文件/</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>每试次 3 s 脑电 → 三类：0 左手(201) / 1 右手(202) / 2 静息(204)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>训练集</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>S01–S06 × 各 5 数据块 × 30 试次 = 900 试次（三类各 300）</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
-      <c r="B9" s="3" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>测试集</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>S07–S08 × 各 2 数据块 × 30 试次 = 120 试次（无 trigger / 无标签）</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>采样率 / 窗</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>250 Hz；每试次 750 点；起点 0,750,…,21750</t>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>250 Hz；每试次 750 点；切分起点 0,750,…,21750</t>
         </is>
       </c>
     </row>
     <row r="11" ht="38" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>通道</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>64 信号通道中取 59 个脑电通道（丢弃 ECG、HEOR、HEOL、VEOU、VEOL）；训练与测试通道顺序一致</t>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>64 信号中取 59 EEG（丢弃 ECG、HEOR、HEOL、VEOU、VEOL）；训练/测试通道序一致</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>预处理硬约束</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>先按试次切分，再滤波/标准化；可学习统计量仅用该折训练集拟合</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>划分与主要结果</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>留一被试交叉验证 6 折（LOSO6）；主要结果 = 逐折嵌套验证集 Acc/召/特；折内读数仅附报</t>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>留一被试交叉验证 6 折（LOSO6）；主要结果=留一被试 Acc/召/特；折内仅附报</t>
         </is>
       </c>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>提交模型</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>QuadFold-59（59 通道从零训练四成员集成）；盲测 CSV 与官方模板 sample_submission.csv 逐行对齐</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>QuadFold-59（59 通道从零四成员集成）；盲测 CSV 对齐官方模板 sample_submission.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>核心指标（摘要）</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Acc 0.5111±0.0657；macro 召回 0.5111；macro 特异 0.7556；运算延迟 1.11 ms；判定延迟 3.00 s（详见 sheet 00/03）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>未使用</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>未使用测试集标签调参；本报告不含自采数据指标</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1"/>
-    <row r="17" ht="22" customHeight="1">
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>完整文字版见交稿包：数据集使用说明.md；官方原文副本见 原始验证数据/官方数据说明.md。</t>
+    <row r="17" ht="22" customHeight="1"/>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>本表即为官方要求的「数据集使用说明」正文（与准/召/特/延迟同文件提交）。官方《数据说明》原文副本见 原始验证数据/官方数据说明.md。</t>
         </is>
       </c>
     </row>
@@ -2399,12 +1768,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="39.4" customWidth="1" min="3" max="3"/>
+    <col width="51.00000000000001" customWidth="1" min="3" max="3"/>
     <col width="38.2" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
   </cols>
@@ -2419,153 +1788,153 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>相对路径</t>
         </is>
       </c>
     </row>
     <row r="5" ht="38" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>嵌套主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>嵌套主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>留一被试主要结果指标 JSON（Acc/召/特/F1/混淆矩阵/六折）</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>原始验证数据/nested_N0_metrics.json</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>盲测提交预测 CSV（官方模板已填 label）</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>原始验证数据/sample_submission.csv</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>同内容内部备份（模型名归档）</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>原始验证数据/submission_QuadFold59.csv</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>嵌套 OOF 概率 / 标签 / 被试</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>留一被试 OOF 概率 / 标签 / 被试</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>原始验证数据/oof_N0/oof_N0_*.npy</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>官方《数据说明》副本</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>原始验证数据/官方数据说明.md</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>本队使用对照摘录</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>原始验证数据/数据说明_使用对照.md</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>验证过程截图 S01–S04</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>验证过程截图 S01–S07</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>验证过程截图/</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>交稿包（邮件附件）</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>交稿/ 或 交稿_离线验证_XH-202610.zip</t>
         </is>
@@ -2573,9 +1942,9 @@
     </row>
     <row r="13" ht="22" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>复算嵌套指标：对 oof_N0_prob.npy 做 argmax，与 oof_N0_y.npy 对照即可复现 sheet 00/01/02。</t>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>复算主要结果：对 oof_N0_prob.npy 做 argmax，与 oof_N0_y.npy 对照即可复现 sheet 00/01/02。</t>
         </is>
       </c>
     </row>
@@ -2593,13 +1962,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A2:F13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="3"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="38.2" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="6"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -2612,192 +1983,186 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>编号</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>文件</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>指定集官方数据核验：目录树、PKL 结构（data 64×22500、ch_names、srate=250）、train 900 / test 120 计数（终端回放）</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>验证过程截图/S01_数据集结构与加载核验.png</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>嵌套验证主结果回放运行：replay_nested.py 现场输出六折 Acc 与 0.511±0.066（终端回放）</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>留一被试主要结果回放：现场输出六折 Acc 与 0.5111±0.0657（终端回放）</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>验证过程截图/S02_嵌套N0指标汇总.png</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>盲测提交 CSV 再生成与比对：predict_submission.py 现场重生成，与提交 CSV 逐行比对（终端回放）</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>盲测提交 CSV 再生成与比对：现场重生成，与提交 CSV 逐行比对（终端回放）</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>验证过程截图/S03_提交CSV再生成与比对.png</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>S04</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>指定集指标独立复算：从 OOF npy 重算 Acc/召/特/F1/CM/六折，逐项对照登记 JSON（终端回放）</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>验证过程截图/S04_独立复算.png</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>提交 CSV 完整性：120 行、表头一致、sample_id 与官方模板逐行对齐、取值合法（终端回放）</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>验证过程截图/S05_提交CSV完整性校验.png</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>S06</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Excel 核心指标与登记 JSON 一致性：程序化读取 00 表单元格对照（终端回放）</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>验证过程截图/S06_Excel与JSON一致性.png</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>交稿包文件 MD5 指纹与运行环境（python/numpy 版本、时间戳；终端回放）</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>验证过程截图/S07_文件指纹与环境.png</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>✅</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="B13" s="9" t="inlineStr">
+    <row r="12"/>
+    <row r="13">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>下列嵌入图便于审阅；原图亦在交稿包 验证过程截图/ 目录。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>注：S07 中 xlsx 自身 MD5 为嵌入本截图前一版的指纹（自引用无法自洽）；交稿包核验以 S07 其余 13 项文件指纹为准。</t>
         </is>
       </c>
     </row>
@@ -2816,13 +2181,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="15.6" customWidth="1" min="2" max="2"/>
-    <col width="63.6" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="6"/>
+    <col width="66.20000000000003" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -2835,74 +2202,74 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>项</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>提交模型</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>QuadFold-59（嵌套主要结果 0.5111 ± 0.0657）</t>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>QuadFold-59（留一被试主要结果 Acc 0.5111±0.0657）</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>主要结果口径</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>留一被试交叉验证 6 折嵌套；折内 0.5580 仅内部参考，不作为对外报告结果</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>主要结果尺子</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>LOSO6 留一被试；禁止用折内 0.5580 作对外主要结果</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>盲测文件</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>sample_submission.csv（官方模板已填 label∈{0,1,2}，120 行）</t>
         </is>
       </c>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>风险否决（归档）</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>备选 8 通道微调方案嵌套 0.540：测试集预测静息类占比约 51%，超出验证集支撑范围，不提交</t>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>备选 8 通道微调栈留一被试 0.5400：测试预测 Rest≈51% 落在验证支撑外，不交</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>纪律</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>超参数与融合权重仅在验证集/嵌套折外选定；测试集标签未用于调参</t>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>超参与融合权仅在验证折外选定；测试标签未用于调参</t>
         </is>
       </c>
     </row>
@@ -2920,12 +2287,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F12"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A2:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="6"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -2938,145 +2308,145 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>核对项</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>期望</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>表内</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>准确率</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="5" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="5" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>召回率 macro</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="7" t="n">
         <v>0.5111</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="7" t="n">
         <v>0.5111</v>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>特异性 macro</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="5" t="n">
         <v>0.7556</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="5" t="n">
         <v>0.7556</v>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>运算延迟</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>1.11 ms</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>判定延迟（指定集）</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>3.00 s</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>OOF 试次数</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="9" t="n">
         <v>900</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="9" t="n">
         <v>900</v>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>盲测 CSV 行数</t>
         </is>
@@ -3087,29 +2457,29 @@
       <c r="D11" s="8" t="n">
         <v>120</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>本报告是否含自采指标</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>✓</t>
         </is>

</xml_diff>